<commit_message>
Use visicart_case_cover as the Visicart home image
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/algovisual-casos.xlsx
+++ b/content/algovisual-casos.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Visicart" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nova Finance App" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shift Analytics Dashboard" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pulse Studio Website" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Terra Coffee Identity" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kite Editorial System" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aether Motion Reel" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Visicart" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Nova Finance App" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Shift Analytics Dashboard" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Pulse Studio Website" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Terra Coffee Identity" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Kite Editorial System" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Aether Motion Reel" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -861,7 +861,7 @@
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>assets/images/visicart-showcase.png</t>
+          <t>assets/images/visicart_case_cover.png</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">

</xml_diff>